<commit_message>
BARS Results: New name for open categories
</commit_message>
<xml_diff>
--- a/local/templates/competitionResults/BARS-Results.xlsx
+++ b/local/templates/competitionResults/BARS-Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/Misc/usaw-owlcms/local/templates/competitionResults/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Library/Application Support/owlcms/64.0.2+quick-start/local/templates/competitionResults/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE48CFCC-CBD2-8E43-BF87-9FCDF56E6BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234591FD-387F-FD4D-A27C-5F446634064C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1460" yWindow="2100" windowWidth="39500" windowHeight="23500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1540" yWindow="660" windowWidth="33020" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -176,15 +176,9 @@
     <t>Junior Women's</t>
   </si>
   <si>
-    <t>Open Men's</t>
-  </si>
-  <si>
     <t>Open M</t>
   </si>
   <si>
-    <t>Open Women's</t>
-  </si>
-  <si>
     <t>Men's Masters (35-39)</t>
   </si>
   <si>
@@ -402,6 +396,12 @@
   </si>
   <si>
     <t>$[VLOOKUP(L2, Validation!$A:$B,2,FALSE)]</t>
+  </si>
+  <si>
+    <t>Men's</t>
+  </si>
+  <si>
+    <t>Women's</t>
   </si>
 </sst>
 </file>
@@ -1134,37 +1134,37 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="H2" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="L2" s="8" t="s">
         <v>81</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1206,34 +1206,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1246,7 +1246,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
@@ -1262,7 +1262,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -1278,7 +1278,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B10" t="s">
         <v>18</v>
@@ -1286,7 +1286,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
@@ -1294,7 +1294,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
         <v>18</v>
@@ -1310,7 +1310,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
         <v>21</v>
@@ -1318,276 +1318,276 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B29" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B30" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B31" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B33" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B34" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B35" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B36" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B37" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B38" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B40" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B41" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B42" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B44" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B45" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B46" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C47" s="9"/>
       <c r="E47" s="9"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C48" s="9"/>
       <c r="E48" s="9"/>

</xml_diff>

<commit_message>
BARS Results: ADAP + WSO age groups
</commit_message>
<xml_diff>
--- a/local/templates/competitionResults/BARS-Results.xlsx
+++ b/local/templates/competitionResults/BARS-Results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Library/Application Support/owlcms/64.0.2+quick-start/local/templates/competitionResults/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/templates/competitionResults/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234591FD-387F-FD4D-A27C-5F446634064C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDABF745-7FFD-1444-ADDE-A78051838F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1540" yWindow="660" windowWidth="33020" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="178">
   <si>
     <t>Lifter Membership ID</t>
   </si>
@@ -323,9 +323,6 @@
     <t>U25 M</t>
   </si>
   <si>
-    <t>U23 M</t>
-  </si>
-  <si>
     <t>U11 M</t>
   </si>
   <si>
@@ -359,9 +356,6 @@
     <t>U25 W</t>
   </si>
   <si>
-    <t>U23 W</t>
-  </si>
-  <si>
     <t>U17 W</t>
   </si>
   <si>
@@ -402,6 +396,252 @@
   </si>
   <si>
     <t>Women's</t>
+  </si>
+  <si>
+    <t>ADAP U25 M</t>
+  </si>
+  <si>
+    <t>ADAP U25 W</t>
+  </si>
+  <si>
+    <t>ADAP U17 M</t>
+  </si>
+  <si>
+    <t>ADAP U17 W</t>
+  </si>
+  <si>
+    <t>ADAP U15 M</t>
+  </si>
+  <si>
+    <t>ADAP U15 W</t>
+  </si>
+  <si>
+    <t>ADAP U13 M</t>
+  </si>
+  <si>
+    <t>ADAP U13 W</t>
+  </si>
+  <si>
+    <t>ADAP U11 M</t>
+  </si>
+  <si>
+    <t>ADAP U11 W</t>
+  </si>
+  <si>
+    <t>ADAP JR M</t>
+  </si>
+  <si>
+    <t>ADAP JR W</t>
+  </si>
+  <si>
+    <t>ADAP M35</t>
+  </si>
+  <si>
+    <t>ADAP W35</t>
+  </si>
+  <si>
+    <t>ADAP M40</t>
+  </si>
+  <si>
+    <t>ADAP W40</t>
+  </si>
+  <si>
+    <t>ADAP M45</t>
+  </si>
+  <si>
+    <t>ADAP W45</t>
+  </si>
+  <si>
+    <t>ADAP M50</t>
+  </si>
+  <si>
+    <t>ADAP W50</t>
+  </si>
+  <si>
+    <t>ADAP M55</t>
+  </si>
+  <si>
+    <t>ADAP W55</t>
+  </si>
+  <si>
+    <t>ADAP M60</t>
+  </si>
+  <si>
+    <t>ADAP W60</t>
+  </si>
+  <si>
+    <t>ADAP M65</t>
+  </si>
+  <si>
+    <t>ADAP W65</t>
+  </si>
+  <si>
+    <t>ADAP M70</t>
+  </si>
+  <si>
+    <t>ADAP W70</t>
+  </si>
+  <si>
+    <t>ADAP M75</t>
+  </si>
+  <si>
+    <t>ADAP W75</t>
+  </si>
+  <si>
+    <t>ADAP M80</t>
+  </si>
+  <si>
+    <t>ADAP W80</t>
+  </si>
+  <si>
+    <t>ADAP M85</t>
+  </si>
+  <si>
+    <t>ADAP W85</t>
+  </si>
+  <si>
+    <t>ADAP M90</t>
+  </si>
+  <si>
+    <t>ADAP W90</t>
+  </si>
+  <si>
+    <t>ADAP M95</t>
+  </si>
+  <si>
+    <t>ADAP W95</t>
+  </si>
+  <si>
+    <t>ADAP M100</t>
+  </si>
+  <si>
+    <t>ADAP W100</t>
+  </si>
+  <si>
+    <t>WSO U25 M</t>
+  </si>
+  <si>
+    <t>WSO U25 W</t>
+  </si>
+  <si>
+    <t>WSO U17 M</t>
+  </si>
+  <si>
+    <t>WSO U17 W</t>
+  </si>
+  <si>
+    <t>WSO U15 M</t>
+  </si>
+  <si>
+    <t>WSO U15 W</t>
+  </si>
+  <si>
+    <t>WSO U13 M</t>
+  </si>
+  <si>
+    <t>WSO U13 W</t>
+  </si>
+  <si>
+    <t>WSO U11 M</t>
+  </si>
+  <si>
+    <t>WSO U11 W</t>
+  </si>
+  <si>
+    <t>WSO JR M</t>
+  </si>
+  <si>
+    <t>WSO JR W</t>
+  </si>
+  <si>
+    <t>WSO M35</t>
+  </si>
+  <si>
+    <t>WSO W35</t>
+  </si>
+  <si>
+    <t>WSO M40</t>
+  </si>
+  <si>
+    <t>WSO W40</t>
+  </si>
+  <si>
+    <t>WSO M45</t>
+  </si>
+  <si>
+    <t>WSO W45</t>
+  </si>
+  <si>
+    <t>WSO M50</t>
+  </si>
+  <si>
+    <t>WSO W50</t>
+  </si>
+  <si>
+    <t>WSO M55</t>
+  </si>
+  <si>
+    <t>WSO W55</t>
+  </si>
+  <si>
+    <t>WSO M60</t>
+  </si>
+  <si>
+    <t>WSO W60</t>
+  </si>
+  <si>
+    <t>WSO M65</t>
+  </si>
+  <si>
+    <t>WSO W65</t>
+  </si>
+  <si>
+    <t>WSO M70</t>
+  </si>
+  <si>
+    <t>WSO W70</t>
+  </si>
+  <si>
+    <t>WSO M75</t>
+  </si>
+  <si>
+    <t>WSO W75</t>
+  </si>
+  <si>
+    <t>WSO M80</t>
+  </si>
+  <si>
+    <t>WSO W80</t>
+  </si>
+  <si>
+    <t>WSO M85</t>
+  </si>
+  <si>
+    <t>WSO W85</t>
+  </si>
+  <si>
+    <t>WSO M90</t>
+  </si>
+  <si>
+    <t>WSO W90</t>
+  </si>
+  <si>
+    <t>WSO M95</t>
+  </si>
+  <si>
+    <t>WSO W95</t>
+  </si>
+  <si>
+    <t>WSO M100</t>
+  </si>
+  <si>
+    <t>WSO W100</t>
+  </si>
+  <si>
+    <t>WSO M</t>
+  </si>
+  <si>
+    <t>WSO W</t>
   </si>
 </sst>
 </file>
@@ -1134,37 +1374,37 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="C2" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="L2" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1197,10 +1437,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="3" width="24.5" customWidth="1"/>
+    <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5" customWidth="1"/>
     <col min="5" max="5" width="26.1640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1209,68 +1451,68 @@
         <v>70</v>
       </c>
       <c r="B1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
@@ -1278,7 +1520,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
         <v>18</v>
@@ -1286,223 +1528,223 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="B15" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>97</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>90</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>96</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>91</v>
+        <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>97</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="B25" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B26" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B27" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B30" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B31" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B32" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B33" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B34" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B35" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B36" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B37" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B38" t="s">
         <v>57</v>
@@ -1510,7 +1752,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B39" t="s">
         <v>59</v>
@@ -1518,7 +1760,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B40" t="s">
         <v>57</v>
@@ -1526,7 +1768,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B41" t="s">
         <v>59</v>
@@ -1534,63 +1776,701 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B42" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>64</v>
-      </c>
-      <c r="B43" t="s">
+      <c r="A43" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B43" s="9" t="s">
         <v>59</v>
       </c>
+      <c r="E43" s="9"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>65</v>
-      </c>
-      <c r="B44" t="s">
+      <c r="A44" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44" s="9" t="s">
         <v>57</v>
       </c>
+      <c r="E44" s="9"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="B45" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="B46" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>99</v>
+      </c>
+      <c r="B48" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>100</v>
+      </c>
+      <c r="B49" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>101</v>
+      </c>
+      <c r="B50" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>102</v>
+      </c>
+      <c r="B51" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>103</v>
+      </c>
+      <c r="B52" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>105</v>
+      </c>
+      <c r="B54" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>106</v>
+      </c>
+      <c r="B55" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>107</v>
+      </c>
+      <c r="B56" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>88</v>
+      </c>
+      <c r="B57" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>89</v>
+      </c>
+      <c r="B58" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>108</v>
+      </c>
+      <c r="B59" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>109</v>
+      </c>
+      <c r="B60" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>110</v>
+      </c>
+      <c r="B61" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>111</v>
+      </c>
+      <c r="B62" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>112</v>
+      </c>
+      <c r="B63" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>113</v>
+      </c>
+      <c r="B64" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>114</v>
+      </c>
+      <c r="B65" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>115</v>
+      </c>
+      <c r="B66" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>116</v>
+      </c>
+      <c r="B67" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>117</v>
+      </c>
+      <c r="B68" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>118</v>
+      </c>
+      <c r="B69" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>119</v>
+      </c>
+      <c r="B70" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>120</v>
+      </c>
+      <c r="B71" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>121</v>
+      </c>
+      <c r="B72" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>122</v>
+      </c>
+      <c r="B73" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>123</v>
+      </c>
+      <c r="B74" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>124</v>
+      </c>
+      <c r="B75" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>125</v>
+      </c>
+      <c r="B76" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B47" s="9" t="s">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>126</v>
+      </c>
+      <c r="B77" t="s">
         <v>59</v>
       </c>
-      <c r="C47" s="9"/>
-      <c r="E47" s="9"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B48" s="9" t="s">
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>127</v>
+      </c>
+      <c r="B78" t="s">
         <v>57</v>
       </c>
-      <c r="C48" s="9"/>
-      <c r="E48" s="9"/>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>128</v>
+      </c>
+      <c r="B79" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>129</v>
+      </c>
+      <c r="B80" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>130</v>
+      </c>
+      <c r="B81" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>131</v>
+      </c>
+      <c r="B82" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>132</v>
+      </c>
+      <c r="B83" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>133</v>
+      </c>
+      <c r="B84" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>134</v>
+      </c>
+      <c r="B85" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>135</v>
+      </c>
+      <c r="B86" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>136</v>
+      </c>
+      <c r="B87" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>137</v>
+      </c>
+      <c r="B88" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>138</v>
+      </c>
+      <c r="B89" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>139</v>
+      </c>
+      <c r="B90" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>140</v>
+      </c>
+      <c r="B91" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>141</v>
+      </c>
+      <c r="B92" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>142</v>
+      </c>
+      <c r="B93" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>143</v>
+      </c>
+      <c r="B94" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>144</v>
+      </c>
+      <c r="B95" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>145</v>
+      </c>
+      <c r="B96" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>146</v>
+      </c>
+      <c r="B97" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>147</v>
+      </c>
+      <c r="B98" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>176</v>
+      </c>
+      <c r="B99" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>177</v>
+      </c>
+      <c r="B100" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>148</v>
+      </c>
+      <c r="B101" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>149</v>
+      </c>
+      <c r="B102" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>150</v>
+      </c>
+      <c r="B103" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>151</v>
+      </c>
+      <c r="B104" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>152</v>
+      </c>
+      <c r="B105" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>153</v>
+      </c>
+      <c r="B106" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>154</v>
+      </c>
+      <c r="B107" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>155</v>
+      </c>
+      <c r="B108" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>156</v>
+      </c>
+      <c r="B109" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>157</v>
+      </c>
+      <c r="B110" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>158</v>
+      </c>
+      <c r="B111" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>159</v>
+      </c>
+      <c r="B112" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>160</v>
+      </c>
+      <c r="B113" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>161</v>
+      </c>
+      <c r="B114" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>162</v>
+      </c>
+      <c r="B115" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>163</v>
+      </c>
+      <c r="B116" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>164</v>
+      </c>
+      <c r="B117" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>165</v>
+      </c>
+      <c r="B118" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>166</v>
+      </c>
+      <c r="B119" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>167</v>
+      </c>
+      <c r="B120" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>168</v>
+      </c>
+      <c r="B121" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>169</v>
+      </c>
+      <c r="B122" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>170</v>
+      </c>
+      <c r="B123" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>171</v>
+      </c>
+      <c r="B124" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>172</v>
+      </c>
+      <c r="B125" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>173</v>
+      </c>
+      <c r="B126" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>174</v>
+      </c>
+      <c r="B127" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>175</v>
+      </c>
+      <c r="B128" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>

</xml_diff>